<commit_message>
chore(catboost): regenerated training artifacts and results
</commit_message>
<xml_diff>
--- a/datasets/Ağaç Yükseklik ve Sayıları.xlsx
+++ b/datasets/Ağaç Yükseklik ve Sayıları.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C09C75-8D00-4EEA-A85D-492C787A93C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A30D3D-F582-4D03-9241-2AEAB6E871FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="13372" xr2:uid="{024612E5-866B-4E60-8589-5D45A3DFAAC3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="42">
   <si>
     <t>WWR</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Ağaç Uzaklığı</t>
   </si>
 </sst>
 </file>
@@ -348,12 +351,45 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -363,9 +399,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -375,44 +408,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -748,205 +751,229 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CA55737-C241-4759-9795-464A010AFFA9}">
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:Z13"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="3" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="9" t="s">
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="15"/>
-      <c r="T1" s="15"/>
-      <c r="U1" s="16" t="s">
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="V1" s="17"/>
+      <c r="Z1" s="15"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="3" t="s">
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="9" t="s">
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="16" t="s">
+      <c r="O2" s="20"/>
+      <c r="P2" s="20"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="20"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="17"/>
+      <c r="Z2" s="15"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="3" t="s">
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="9" t="s">
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="11"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
       <c r="Q3" s="20"/>
-      <c r="R3" s="21"/>
+      <c r="R3" s="20"/>
       <c r="S3" s="21"/>
-      <c r="T3" s="21"/>
-      <c r="U3" s="16" t="s">
+      <c r="T3" s="24"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="V3" s="17"/>
+      <c r="Z3" s="15"/>
     </row>
-    <row r="4" spans="1:22" ht="26.6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:26" ht="26.6" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="L4" s="12" t="s">
+      <c r="M4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="O4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="P4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="Q4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="R4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="P4" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="22" t="s">
+      <c r="S4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="T4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="R4" s="22" t="s">
+      <c r="U4" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S4" s="22" t="s">
+      <c r="V4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="W4" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="T4" s="22" t="s">
+      <c r="X4" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="U4" s="22" t="s">
+      <c r="Y4" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="V4" s="22" t="s">
+      <c r="Z4" s="8" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="12">
-        <v>1</v>
-      </c>
-      <c r="C5" s="12">
+      <c r="B5" s="3">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3">
         <v>5</v>
       </c>
-      <c r="D5" s="12">
-        <v>2</v>
-      </c>
-      <c r="E5" s="13">
+      <c r="E5" s="3">
+        <v>2</v>
+      </c>
+      <c r="F5" s="4">
         <v>4</v>
       </c>
-      <c r="F5" s="13">
+      <c r="G5" s="4">
         <v>0.26200000000000001</v>
       </c>
-      <c r="G5" s="24" t="s">
+      <c r="H5" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="2">
-        <v>0</v>
-      </c>
-      <c r="I5" s="2">
+      <c r="I5" s="10">
         <v>0</v>
       </c>
       <c r="J5" s="2">
@@ -955,66 +982,78 @@
       <c r="K5" s="2">
         <v>0</v>
       </c>
-      <c r="L5" s="13">
+      <c r="L5" s="2">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4">
         <v>3.5</v>
       </c>
-      <c r="M5" s="13">
-        <v>0</v>
-      </c>
-      <c r="N5" s="13">
-        <v>0</v>
-      </c>
-      <c r="O5" s="13">
-        <v>0</v>
-      </c>
-      <c r="P5" s="13">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="22" t="s">
+      <c r="O5" s="4">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>0</v>
+      </c>
+      <c r="R5" s="4">
+        <v>0</v>
+      </c>
+      <c r="S5" s="4">
+        <v>0</v>
+      </c>
+      <c r="T5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="R5" s="22">
+      <c r="U5" s="8">
         <v>4.5</v>
       </c>
-      <c r="S5" s="22">
+      <c r="V5" s="8">
+        <v>5</v>
+      </c>
+      <c r="W5" s="8">
         <v>9</v>
       </c>
-      <c r="T5" s="22">
-        <v>1</v>
-      </c>
-      <c r="U5" s="23">
-        <v>1</v>
-      </c>
-      <c r="V5" s="23">
+      <c r="X5" s="8">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="9">
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="3">
         <v>6</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="3">
+        <v>4</v>
+      </c>
+      <c r="D6" s="3">
         <v>5</v>
       </c>
-      <c r="D6" s="12">
-        <v>2</v>
-      </c>
-      <c r="E6" s="13">
-        <v>2</v>
-      </c>
-      <c r="F6" s="13">
+      <c r="E6" s="3">
+        <v>2</v>
+      </c>
+      <c r="F6" s="4">
+        <v>2</v>
+      </c>
+      <c r="G6" s="4">
         <v>0.26200000000000001</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="H6" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="H6" s="2">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2">
+      <c r="I6" s="10">
         <v>0</v>
       </c>
       <c r="J6" s="2">
@@ -1023,406 +1062,478 @@
       <c r="K6" s="2">
         <v>0</v>
       </c>
-      <c r="L6" s="13">
+      <c r="L6" s="2">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0</v>
+      </c>
+      <c r="N6" s="4">
         <v>9.5</v>
       </c>
-      <c r="M6" s="13">
-        <v>0</v>
-      </c>
-      <c r="N6" s="13">
-        <v>0</v>
-      </c>
-      <c r="O6" s="13">
-        <v>0</v>
-      </c>
-      <c r="P6" s="13">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="22" t="s">
+      <c r="O6" s="4">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>0</v>
+      </c>
+      <c r="R6" s="4">
+        <v>0</v>
+      </c>
+      <c r="S6" s="4">
+        <v>0</v>
+      </c>
+      <c r="T6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="R6" s="22">
+      <c r="U6" s="8">
         <v>16.5</v>
       </c>
-      <c r="S6" s="22">
+      <c r="V6" s="8">
+        <v>5</v>
+      </c>
+      <c r="W6" s="8">
         <v>9</v>
       </c>
-      <c r="T6" s="22">
-        <v>1</v>
-      </c>
-      <c r="U6" s="23">
-        <v>1</v>
-      </c>
-      <c r="V6" s="23">
+      <c r="X6" s="8">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="9">
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="12">
-        <v>1</v>
-      </c>
-      <c r="C7" s="12">
+      <c r="B7" s="3">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3">
         <v>9</v>
       </c>
-      <c r="D7" s="12">
-        <v>2</v>
-      </c>
-      <c r="E7" s="13">
+      <c r="E7" s="3">
+        <v>2</v>
+      </c>
+      <c r="F7" s="4">
         <v>3</v>
       </c>
-      <c r="F7" s="13">
+      <c r="G7" s="4">
         <v>0.34899999999999998</v>
       </c>
-      <c r="G7" s="2">
-        <v>1</v>
-      </c>
       <c r="H7" s="2">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2">
         <v>15</v>
       </c>
-      <c r="I7" s="2">
-        <v>1</v>
-      </c>
       <c r="J7" s="2">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="K7" s="2">
+        <v>1</v>
+      </c>
+      <c r="L7" s="2">
+        <v>1</v>
+      </c>
+      <c r="M7" s="2">
         <v>0.111</v>
       </c>
-      <c r="L7" s="13">
+      <c r="N7" s="4">
         <v>3.5</v>
       </c>
-      <c r="M7" s="13">
+      <c r="O7" s="4">
+        <v>11.5</v>
+      </c>
+      <c r="P7" s="4">
         <v>9</v>
       </c>
-      <c r="N7" s="13">
-        <v>1</v>
-      </c>
-      <c r="O7" s="13">
-        <v>2</v>
-      </c>
-      <c r="P7" s="13">
+      <c r="Q7" s="4">
+        <v>1</v>
+      </c>
+      <c r="R7" s="4">
+        <v>2</v>
+      </c>
+      <c r="S7" s="4">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q7" s="22" t="s">
+      <c r="T7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="R7" s="22">
+      <c r="U7" s="8">
         <v>31.5</v>
       </c>
-      <c r="S7" s="22">
+      <c r="V7" s="8">
+        <v>5</v>
+      </c>
+      <c r="W7" s="8">
         <v>9</v>
       </c>
-      <c r="T7" s="22">
-        <v>1</v>
-      </c>
-      <c r="U7" s="23">
-        <v>0</v>
-      </c>
-      <c r="V7" s="23">
+      <c r="X7" s="8">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="9">
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="3">
+        <v>6</v>
+      </c>
+      <c r="D8" s="3">
         <v>9</v>
       </c>
-      <c r="D8" s="12">
-        <v>2</v>
-      </c>
-      <c r="E8" s="13">
+      <c r="E8" s="3">
+        <v>2</v>
+      </c>
+      <c r="F8" s="4">
         <v>3</v>
       </c>
-      <c r="F8" s="13">
+      <c r="G8" s="4">
         <v>0.34899999999999998</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8" s="2">
         <v>4.5</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I8" s="2">
         <v>15</v>
       </c>
-      <c r="I8" s="2">
-        <v>1</v>
-      </c>
       <c r="J8" s="2">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="K8" s="2">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2">
         <v>0.16700000000000001</v>
       </c>
-      <c r="L8" s="13">
+      <c r="N8" s="4">
         <v>9.5</v>
       </c>
-      <c r="M8" s="13">
+      <c r="O8" s="4">
+        <v>11.5</v>
+      </c>
+      <c r="P8" s="4">
         <v>9</v>
       </c>
-      <c r="N8" s="13">
-        <v>1</v>
-      </c>
-      <c r="O8" s="13">
-        <v>1</v>
-      </c>
-      <c r="P8" s="13">
+      <c r="Q8" s="4">
+        <v>1</v>
+      </c>
+      <c r="R8" s="4">
+        <v>1</v>
+      </c>
+      <c r="S8" s="4">
         <v>0.67200000000000004</v>
       </c>
-      <c r="Q8" s="22" t="s">
+      <c r="T8" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="R8" s="22">
+      <c r="U8" s="8">
         <v>4.5</v>
       </c>
-      <c r="S8" s="22">
+      <c r="V8" s="8">
+        <v>3</v>
+      </c>
+      <c r="W8" s="8">
         <v>18</v>
       </c>
-      <c r="T8" s="22">
-        <v>1</v>
-      </c>
-      <c r="U8" s="23">
-        <v>2</v>
-      </c>
-      <c r="V8" s="23">
+      <c r="X8" s="8">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="9">
+        <v>2</v>
+      </c>
+      <c r="Z8" s="9">
         <v>0.443</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="12">
-        <v>1</v>
-      </c>
-      <c r="C9" s="12">
+      <c r="B9" s="3">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3">
         <v>9</v>
       </c>
-      <c r="D9" s="12">
-        <v>1</v>
-      </c>
-      <c r="E9" s="13">
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" s="4">
         <v>3</v>
       </c>
-      <c r="F9" s="13">
+      <c r="G9" s="4">
         <v>0.26200000000000001</v>
       </c>
-      <c r="G9" s="2">
-        <v>1</v>
-      </c>
       <c r="H9" s="2">
+        <v>1</v>
+      </c>
+      <c r="I9" s="2">
+        <v>7</v>
+      </c>
+      <c r="J9" s="2">
         <v>10</v>
       </c>
-      <c r="I9" s="2">
-        <v>2</v>
-      </c>
-      <c r="J9" s="2">
-        <v>2</v>
-      </c>
       <c r="K9" s="2">
+        <v>2</v>
+      </c>
+      <c r="L9" s="2">
+        <v>2</v>
+      </c>
+      <c r="M9" s="2">
         <v>0.34699999999999998</v>
       </c>
-      <c r="L9" s="13">
+      <c r="N9" s="4">
         <v>3.5</v>
       </c>
-      <c r="M9" s="13">
+      <c r="O9" s="4">
+        <v>4.5</v>
+      </c>
+      <c r="P9" s="4">
         <v>13</v>
       </c>
-      <c r="N9" s="13">
-        <v>2</v>
-      </c>
-      <c r="O9" s="13">
+      <c r="Q9" s="4">
+        <v>2</v>
+      </c>
+      <c r="R9" s="4">
         <v>3</v>
       </c>
-      <c r="P9" s="13">
+      <c r="S9" s="4">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q9" s="22" t="s">
+      <c r="T9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="R9" s="22">
+      <c r="U9" s="8">
         <v>16.5</v>
       </c>
-      <c r="S9" s="22">
+      <c r="V9" s="8">
+        <v>3</v>
+      </c>
+      <c r="W9" s="8">
         <v>18</v>
       </c>
-      <c r="T9" s="22">
-        <v>1</v>
-      </c>
-      <c r="U9" s="23">
-        <v>0</v>
-      </c>
-      <c r="V9" s="23">
+      <c r="X9" s="8">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="9">
         <v>0.443</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="3">
         <v>6</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="3">
+        <v>6</v>
+      </c>
+      <c r="D10" s="3">
         <v>9</v>
       </c>
-      <c r="D10" s="12">
-        <v>1</v>
-      </c>
-      <c r="E10" s="13">
-        <v>2</v>
-      </c>
-      <c r="F10" s="13">
+      <c r="E10" s="3">
+        <v>1</v>
+      </c>
+      <c r="F10" s="4">
+        <v>2</v>
+      </c>
+      <c r="G10" s="4">
         <v>0.26200000000000001</v>
       </c>
-      <c r="G10" s="2">
+      <c r="H10" s="2">
         <v>4.5</v>
       </c>
-      <c r="H10" s="2">
+      <c r="I10" s="2">
+        <v>7</v>
+      </c>
+      <c r="J10" s="2">
         <v>20</v>
       </c>
-      <c r="I10" s="2">
-        <v>2</v>
-      </c>
-      <c r="J10" s="2">
-        <v>2</v>
-      </c>
       <c r="K10" s="2">
+        <v>2</v>
+      </c>
+      <c r="L10" s="2">
+        <v>2</v>
+      </c>
+      <c r="M10" s="2">
         <v>0.16700000000000001</v>
       </c>
-      <c r="L10" s="13">
+      <c r="N10" s="4">
         <v>9.5</v>
       </c>
-      <c r="M10" s="13">
+      <c r="O10" s="4">
+        <v>4.5</v>
+      </c>
+      <c r="P10" s="4">
         <v>13</v>
       </c>
-      <c r="N10" s="13">
-        <v>2</v>
-      </c>
-      <c r="O10" s="13">
-        <v>2</v>
-      </c>
-      <c r="P10" s="13">
+      <c r="Q10" s="4">
+        <v>2</v>
+      </c>
+      <c r="R10" s="4">
+        <v>2</v>
+      </c>
+      <c r="S10" s="4">
         <v>0.67200000000000004</v>
       </c>
-      <c r="Q10" s="22" t="s">
+      <c r="T10" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="R10" s="22">
+      <c r="U10" s="8">
         <v>31.5</v>
       </c>
-      <c r="S10" s="22">
+      <c r="V10" s="8">
+        <v>3</v>
+      </c>
+      <c r="W10" s="8">
         <v>18</v>
       </c>
-      <c r="T10" s="22">
-        <v>1</v>
-      </c>
-      <c r="U10" s="23">
-        <v>0</v>
-      </c>
-      <c r="V10" s="23">
+      <c r="X10" s="8">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="9">
         <v>0.443</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="12">
-        <v>1</v>
-      </c>
-      <c r="C11" s="12">
-        <v>0</v>
-      </c>
-      <c r="D11" s="12">
-        <v>0</v>
-      </c>
-      <c r="E11" s="13">
-        <v>0</v>
-      </c>
-      <c r="F11" s="13">
-        <v>0</v>
-      </c>
-      <c r="G11" s="24">
-        <v>1</v>
-      </c>
-      <c r="H11" s="2">
+      <c r="B11" s="3">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11" s="10">
+        <v>1</v>
+      </c>
+      <c r="I11" s="10">
         <v>10</v>
       </c>
-      <c r="I11" s="2">
-        <v>2</v>
-      </c>
       <c r="J11" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K11" s="2">
+        <v>2</v>
+      </c>
+      <c r="L11" s="2">
+        <v>2</v>
+      </c>
+      <c r="M11" s="2">
         <v>0.33300000000000002</v>
       </c>
-      <c r="L11" s="13">
+      <c r="N11" s="4">
         <v>3.5</v>
       </c>
-      <c r="M11" s="13">
-        <v>0</v>
-      </c>
-      <c r="N11" s="13">
-        <v>0</v>
-      </c>
-      <c r="O11" s="13">
-        <v>0</v>
-      </c>
-      <c r="P11" s="13">
+      <c r="O11" s="4">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4">
+        <v>0</v>
+      </c>
+      <c r="R11" s="4">
+        <v>0</v>
+      </c>
+      <c r="S11" s="4">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q11" s="22" t="s">
+      <c r="T11" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="R11" s="22">
+      <c r="U11" s="8">
         <v>4.5</v>
       </c>
-      <c r="S11" s="22">
-        <v>0</v>
-      </c>
-      <c r="T11" s="22">
-        <v>0</v>
-      </c>
-      <c r="U11" s="23">
-        <v>1</v>
-      </c>
-      <c r="V11" s="23">
+      <c r="V11" s="8">
+        <v>3</v>
+      </c>
+      <c r="W11" s="8">
+        <v>0</v>
+      </c>
+      <c r="X11" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="9">
         <v>0.41399999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="12">
-        <v>6</v>
-      </c>
-      <c r="C12" s="12">
-        <v>0</v>
-      </c>
-      <c r="D12" s="12">
-        <v>0</v>
-      </c>
-      <c r="E12" s="13">
-        <v>0</v>
-      </c>
-      <c r="F12" s="13">
-        <v>0</v>
-      </c>
-      <c r="G12" s="24" t="s">
+      <c r="B12" s="3">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="2">
-        <v>0</v>
-      </c>
-      <c r="I12" s="2">
+      <c r="I12" s="10">
         <v>0</v>
       </c>
       <c r="J12" s="2">
@@ -1431,92 +1542,110 @@
       <c r="K12" s="2">
         <v>0</v>
       </c>
-      <c r="L12" s="13">
+      <c r="L12" s="2">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0</v>
+      </c>
+      <c r="N12" s="4">
         <v>9.5</v>
       </c>
-      <c r="M12" s="13">
-        <v>0</v>
-      </c>
-      <c r="N12" s="13">
-        <v>0</v>
-      </c>
-      <c r="O12" s="13">
-        <v>0</v>
-      </c>
-      <c r="P12" s="13" t="s">
+      <c r="O12" s="4">
+        <v>0</v>
+      </c>
+      <c r="P12" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4">
+        <v>0</v>
+      </c>
+      <c r="R12" s="4">
+        <v>0</v>
+      </c>
+      <c r="S12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Q12" s="22" t="s">
+      <c r="T12" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="R12" s="22">
+      <c r="U12" s="8">
         <v>16.5</v>
       </c>
-      <c r="S12" s="22">
-        <v>0</v>
-      </c>
-      <c r="T12" s="22">
-        <v>0</v>
-      </c>
-      <c r="U12" s="23">
-        <v>0</v>
-      </c>
-      <c r="V12" s="23">
+      <c r="V12" s="8">
+        <v>3</v>
+      </c>
+      <c r="W12" s="8">
+        <v>0</v>
+      </c>
+      <c r="X12" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="9">
         <v>0.41399999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="22" t="s">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="A13" s="16"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="17"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="17"/>
+      <c r="S13" s="18"/>
+      <c r="T13" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="R13" s="22">
+      <c r="U13" s="8">
         <v>31.5</v>
       </c>
-      <c r="S13" s="22">
-        <v>0</v>
-      </c>
-      <c r="T13" s="22">
-        <v>0</v>
-      </c>
-      <c r="U13" s="23">
-        <v>0</v>
-      </c>
-      <c r="V13" s="23" t="s">
+      <c r="V13" s="8">
+        <v>3</v>
+      </c>
+      <c r="W13" s="8">
+        <v>0</v>
+      </c>
+      <c r="X13" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="9" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="A13:P13"/>
-    <mergeCell ref="L1:P1"/>
-    <mergeCell ref="L2:P2"/>
-    <mergeCell ref="L3:P3"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="Q1:Q3"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="U2:V2"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="H3:M3"/>
+    <mergeCell ref="Y3:Z3"/>
+    <mergeCell ref="A13:S13"/>
+    <mergeCell ref="N1:S1"/>
+    <mergeCell ref="N2:S2"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="T1:T3"/>
+    <mergeCell ref="Y1:Z1"/>
+    <mergeCell ref="Y2:Z2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>